<commit_message>
Excel v2: reverse game column order + complete box scores + roster fix
ユーザー要望に基づく修正：
1. ゲーム列順を逆転：左から G3(5/8新) → G2(5/6) → G1(5/4旧)
2. ボックススコアを大幅充実（複数ソース照合：ESPN / NBA.com /
   RotoWire / CBS Sports / FanDuel Research / Posting and Toasting /
   Liberty Ballers / SI / Yahoo Sports）
3. ロースター修正：
   - Cameron Payne 削除（4月に76ersから契約解除＋ハム筋挫傷）
   - Dalen Terry 追加（10日間契約から本契約に昇格）
   - Murray State 表記誤り（旧マレーシア州立大→マレー州立大）はPayne
     削除によって解消

確認できないセルは "—" 表記（推測なし）。完全DNPは "DNP"、
インアクティブ/負傷は "OUT" として6セルマージで明示。

主要な追加・確定スタッツ：
- Brunson G3: 38分33点・3-8 3PT・9アシスト5リバ確定
- Bridges G1: 27分17点・3-5 3PT・5アシスト2リバ（旧3アシストから訂正）
- Anunoby G2: 37分24点・2-7 3PT（試合終盤ハム負傷退場）
- Hart G3: 40分12点・0-4 3PT・3アシスト11リバ
- Robinson G3: 19分・3-4 FT・OREB 2本・チームは在ベンチ時+16
- Maxey G2: 47分26点・1-6 3PT・6アシスト3リバ（9-22 FG）
- George G3: 38分15点・3 3PT（Q1で6-9から残り0-9）
- Edgecombe G2: 40分17点・3-7 3PT・3アシスト5リバ
- Embiid G3: 35分18点・0-4 3PT・5アシスト6リバ・3ブロック（復帰戦）
- Bona G1: 4分0点・5ファウル（3:47で記録タイ）
- Terry G3: 短時間出場（具体的スタッツ未確認）
</commit_message>
<xml_diff>
--- a/nba_stats_PHI_NYK_20260510.xlsx
+++ b/nba_stats_PHI_NYK_20260510.xlsx
@@ -587,7 +587,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>2026 NBAプレーオフ 第2回戦・第4戦  フィラデルフィア・76ers @ ニューヨーク・ニックス  2026/5/10(現地)・JST 5/11 4:30 タップオフ ／ シリーズ 3勝1敗（NYKリード）</t>
+          <t>2026 NBAプレーオフ 第2回戦・第4戦  フィラデルフィア・76ers @ ニューヨーク・ニックス  2026/5/10(現地)・JST 5/11 4:30 タップオフ ／ シリーズ 3勝0敗（NYKリード）  ※ G列順は新しい試合（G3=5/8）が左</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>G1 5/4 ○137-98 vs PHI (MSG)</t>
+          <t>シリーズ第3戦 5/8 ○108-94 @PHI</t>
         </is>
       </c>
       <c r="J3" s="5" t="n"/>
@@ -668,7 +668,7 @@
       <c r="N3" s="5" t="n"/>
       <c r="O3" s="4" t="inlineStr">
         <is>
-          <t>G2 5/6 ○108-102 vs PHI (MSG)</t>
+          <t>シリーズ第2戦 5/6 ○108-102 vs PHI</t>
         </is>
       </c>
       <c r="P3" s="5" t="n"/>
@@ -678,7 +678,7 @@
       <c r="T3" s="5" t="n"/>
       <c r="U3" s="4" t="inlineStr">
         <is>
-          <t>G3 5/8 ○108-94 @PHI</t>
+          <t>シリーズ第1戦 5/4 ○137-98 vs PHI</t>
         </is>
       </c>
       <c r="V3" s="5" t="n"/>
@@ -837,22 +837,22 @@
         </is>
       </c>
       <c r="I5" s="10" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="J5" s="10" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="K5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="L5" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M5" s="10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N5" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O5" s="10" t="n">
         <v>41</v>
@@ -860,15 +860,11 @@
       <c r="P5" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="Q5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="S5" s="10" t="n">
         <v>6</v>
@@ -877,26 +873,22 @@
         <v>1</v>
       </c>
       <c r="U5" s="10" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="V5" s="10" t="n">
-        <v>33</v>
-      </c>
-      <c r="W5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X5" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>35</v>
+      </c>
+      <c r="W5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="X5" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="Y5" s="10" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="Z5" s="10" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
@@ -937,22 +929,22 @@
         </is>
       </c>
       <c r="I6" s="14" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="K6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="14" t="n">
         <v>3</v>
-      </c>
-      <c r="L6" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="M6" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="N6" s="14" t="n">
-        <v>2</v>
       </c>
       <c r="O6" s="14" t="n">
         <v>38</v>
@@ -962,41 +954,39 @@
       </c>
       <c r="Q6" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R6" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S6" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T6" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T6" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="U6" s="14" t="n">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="V6" s="14" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="W6" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="X6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="Z6" s="14" t="n">
         <v>2</v>
-      </c>
-      <c r="X6" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="Y6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z6" s="14" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -1036,68 +1026,52 @@
           <t>【Q/右ハム】インディアナ大出身。3&amp;D駒、G3欠場</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>18</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="I7" s="15" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="n"/>
+      <c r="K7" s="16" t="n"/>
+      <c r="L7" s="16" t="n"/>
+      <c r="M7" s="16" t="n"/>
+      <c r="N7" s="16" t="n"/>
       <c r="O7" s="10" t="n">
         <v>37</v>
       </c>
       <c r="P7" s="10" t="n">
         <v>24</v>
       </c>
-      <c r="Q7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="R7" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="S7" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="T7" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="U7" s="15" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="V7" s="16" t="n"/>
-      <c r="W7" s="16" t="n"/>
-      <c r="X7" s="16" t="n"/>
-      <c r="Y7" s="16" t="n"/>
-      <c r="Z7" s="16" t="n"/>
+      <c r="U7" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="V7" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="W7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="X7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="10" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="8" ht="28" customHeight="1">
       <c r="A8" s="11" t="n">
@@ -1137,22 +1111,22 @@
         </is>
       </c>
       <c r="I8" s="14" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="J8" s="14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L8" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M8" s="14" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N8" s="14" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="O8" s="14" t="n">
         <v>44</v>
@@ -1172,31 +1146,23 @@
       <c r="T8" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="U8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U8" s="14" t="n">
+        <v>26</v>
       </c>
       <c r="V8" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="W8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y8" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="W8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X8" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y8" s="14" t="n">
+        <v>6</v>
       </c>
       <c r="Z8" s="14" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
@@ -1237,22 +1203,22 @@
         </is>
       </c>
       <c r="I9" s="10" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="J9" s="10" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="K9" s="10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L9" s="10" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="M9" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N9" s="10" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="O9" s="10" t="n">
         <v>27</v>
@@ -1273,22 +1239,22 @@
         <v>10</v>
       </c>
       <c r="U9" s="10" t="n">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="V9" s="10" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="W9" s="10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="X9" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="Y9" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Z9" s="10" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
@@ -1329,10 +1295,10 @@
         </is>
       </c>
       <c r="I10" s="14" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="J10" s="14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K10" s="14" t="n">
         <v>0</v>
@@ -1340,11 +1306,13 @@
       <c r="L10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="M10" s="14" t="n">
-        <v>1</v>
+      <c r="M10" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="N10" s="14" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O10" s="17" t="inlineStr">
         <is>
@@ -1357,12 +1325,10 @@
       <c r="S10" s="18" t="n"/>
       <c r="T10" s="18" t="n"/>
       <c r="U10" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="V10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="V10" s="14" t="n">
+        <v>2</v>
       </c>
       <c r="W10" s="14" t="n">
         <v>0</v>
@@ -1370,15 +1336,11 @@
       <c r="X10" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="Y10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z10" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Y10" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="14" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -1418,34 +1380,24 @@
           <t>ウェストバージニア大出身。Deuceの愛称、対人守備の切り札</t>
         </is>
       </c>
-      <c r="I11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I11" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M11" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="N11" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O11" s="10" t="n">
@@ -1466,34 +1418,24 @@
       <c r="T11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="U11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y11" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U11" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="V11" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="W11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="X11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y11" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="Z11" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1536,93 +1478,69 @@
       </c>
       <c r="I12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O12" s="14" t="n">
+        <v>7</v>
+      </c>
+      <c r="P12" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="S12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="T12" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="14" t="n">
+        <v>9</v>
+      </c>
+      <c r="V12" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="W12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="X12" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z12" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z12" s="14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
@@ -1662,83 +1580,67 @@
           <t>ウィチタ州立大出身。3P39%超のシューター</t>
         </is>
       </c>
-      <c r="I13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I13" s="10" t="n">
+        <v>26</v>
       </c>
       <c r="J13" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="K13" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="O13" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="P13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="R13" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S13" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="T13" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U13" s="10" t="n">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="V13" s="10" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="W13" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X13" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="Y13" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Y13" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="Z13" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
@@ -1780,85 +1682,67 @@
       </c>
       <c r="I14" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="n">
+        <v>4</v>
       </c>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="N14" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="O14" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="P14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q14" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="S14" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T14" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="U14" s="14" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="V14" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="W14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X14" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="W14" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X14" s="14" t="n">
+        <v>3</v>
       </c>
       <c r="Y14" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="Z14" s="14" t="n">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="Z14" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
@@ -1898,36 +1782,16 @@
           <t>ドイツ出身の若手C。第3ユニットの控え</t>
         </is>
       </c>
-      <c r="I15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="I15" s="15" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="J15" s="16" t="n"/>
+      <c r="K15" s="16" t="n"/>
+      <c r="L15" s="16" t="n"/>
+      <c r="M15" s="16" t="n"/>
+      <c r="N15" s="16" t="n"/>
       <c r="O15" s="10" t="n">
         <v>7</v>
       </c>
@@ -1942,41 +1806,31 @@
       </c>
       <c r="S15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="T15" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="U15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U15" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="V15" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="W15" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="Y15" s="10" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z15" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z15" s="10" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
@@ -2013,7 +1867,7 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>マーケット大出身2年目PG。プレーオフ出場機会限定的</t>
+          <t>マーケット大出身2年目PG。Gリーグで2桁アシスト連発</t>
         </is>
       </c>
       <c r="I16" s="17" t="inlineStr">
@@ -2036,16 +1890,32 @@
       <c r="R16" s="18" t="n"/>
       <c r="S16" s="18" t="n"/>
       <c r="T16" s="18" t="n"/>
-      <c r="U16" s="17" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="V16" s="18" t="n"/>
-      <c r="W16" s="18" t="n"/>
-      <c r="X16" s="18" t="n"/>
-      <c r="Y16" s="18" t="n"/>
-      <c r="Z16" s="18" t="n"/>
+      <c r="U16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V16" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="W16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y16" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z16" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="28" customHeight="1">
       <c r="A17" s="7" t="n">
@@ -2104,16 +1974,32 @@
       <c r="R17" s="16" t="n"/>
       <c r="S17" s="16" t="n"/>
       <c r="T17" s="16" t="n"/>
-      <c r="U17" s="15" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="V17" s="16" t="n"/>
-      <c r="W17" s="16" t="n"/>
-      <c r="X17" s="16" t="n"/>
-      <c r="Y17" s="16" t="n"/>
-      <c r="Z17" s="16" t="n"/>
+      <c r="U17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="V17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="W17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="X17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z17" s="10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" ht="28" customHeight="1">
       <c r="A18" s="11" t="n">
@@ -2172,16 +2058,24 @@
       <c r="R18" s="18" t="n"/>
       <c r="S18" s="18" t="n"/>
       <c r="T18" s="18" t="n"/>
-      <c r="U18" s="17" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="V18" s="18" t="n"/>
-      <c r="W18" s="18" t="n"/>
-      <c r="X18" s="18" t="n"/>
-      <c r="Y18" s="18" t="n"/>
-      <c r="Z18" s="18" t="n"/>
+      <c r="U18" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="V18" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="W18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="X18" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y18" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z18" s="14" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="19" ht="28" customHeight="1">
       <c r="A19" s="7" t="n">
@@ -2217,7 +2111,7 @@
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>ベイラー大出身。2/13に加入、フロントコート補強</t>
+          <t>ベイラー大出身。2/13にスパーズから加入、フロントコート補強</t>
         </is>
       </c>
       <c r="I19" s="15" t="inlineStr">
@@ -2230,16 +2124,24 @@
       <c r="L19" s="16" t="n"/>
       <c r="M19" s="16" t="n"/>
       <c r="N19" s="16" t="n"/>
-      <c r="O19" s="15" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="P19" s="16" t="n"/>
-      <c r="Q19" s="16" t="n"/>
-      <c r="R19" s="16" t="n"/>
-      <c r="S19" s="16" t="n"/>
-      <c r="T19" s="16" t="n"/>
+      <c r="O19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="10" t="n">
+        <v>0</v>
+      </c>
       <c r="U19" s="15" t="inlineStr">
         <is>
           <t>DNP</t>
@@ -2318,7 +2220,7 @@
       </c>
       <c r="I22" s="21" t="inlineStr">
         <is>
-          <t>G1 5/4 ●98-137 @NYK</t>
+          <t>シリーズ第3戦 5/8 ●94-108 vs NYK</t>
         </is>
       </c>
       <c r="J22" s="22" t="n"/>
@@ -2328,7 +2230,7 @@
       <c r="N22" s="22" t="n"/>
       <c r="O22" s="21" t="inlineStr">
         <is>
-          <t>G2 5/6 ●102-108 @NYK (Embiid OUT)</t>
+          <t>シリーズ第2戦 5/6 ●102-108 @NYK</t>
         </is>
       </c>
       <c r="P22" s="22" t="n"/>
@@ -2338,7 +2240,7 @@
       <c r="T22" s="22" t="n"/>
       <c r="U22" s="21" t="inlineStr">
         <is>
-          <t>G3 5/8 ●94-108 vs NYK (Embiid復帰)</t>
+          <t>シリーズ第1戦 5/4 ●98-137 @NYK</t>
         </is>
       </c>
       <c r="V22" s="22" t="n"/>
@@ -2497,22 +2399,22 @@
         </is>
       </c>
       <c r="I24" s="10" t="n">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="J24" s="10" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K24" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" s="10" t="n">
         <v>3</v>
       </c>
       <c r="M24" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="N24" s="10" t="n">
         <v>2</v>
-      </c>
-      <c r="N24" s="10" t="n">
-        <v>3</v>
       </c>
       <c r="O24" s="10" t="n">
         <v>47</v>
@@ -2520,39 +2422,35 @@
       <c r="P24" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="Q24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R24" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q24" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R24" s="10" t="n">
+        <v>6</v>
       </c>
       <c r="S24" s="10" t="n">
         <v>6</v>
       </c>
       <c r="T24" s="10" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="U24" s="10" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="V24" s="10" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="W24" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X24" s="10" t="n">
         <v>3</v>
       </c>
       <c r="Y24" s="10" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="Z24" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" ht="28" customHeight="1">
@@ -2592,41 +2490,41 @@
           <t>ベイラー大出身、新人王最終候補のバハマ出身ルーキー</t>
         </is>
       </c>
-      <c r="I25" s="14" t="n">
-        <v>28</v>
+      <c r="I25" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="J25" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="K25" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="L25" s="14" t="n">
-        <v>5</v>
+        <v>11</v>
+      </c>
+      <c r="K25" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M25" s="14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N25" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="O25" s="14" t="n">
+        <v>40</v>
       </c>
       <c r="P25" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="Q25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="Q25" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="R25" s="14" t="n">
+        <v>7</v>
       </c>
       <c r="S25" s="14" t="n">
         <v>3</v>
@@ -2634,29 +2532,23 @@
       <c r="T25" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="U25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U25" s="14" t="n">
+        <v>28</v>
       </c>
       <c r="V25" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="W25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X25" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>12</v>
+      </c>
+      <c r="W25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="X25" s="14" t="n">
+        <v>5</v>
       </c>
       <c r="Y25" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="Z25" s="14" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
@@ -2696,75 +2588,61 @@
           <t>カンザス大出身、爆発力のあるアスレチック系3&amp;D</t>
         </is>
       </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I26" s="10" t="n">
+        <v>36</v>
       </c>
       <c r="J26" s="10" t="n">
-        <v>12</v>
-      </c>
-      <c r="K26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>22</v>
+      </c>
+      <c r="K26" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="10" t="n">
+        <v>5</v>
       </c>
       <c r="M26" s="10" t="n">
         <v>1</v>
       </c>
       <c r="N26" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="O26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="O26" s="10" t="n">
+        <v>40</v>
       </c>
       <c r="P26" s="10" t="n">
         <v>19</v>
       </c>
-      <c r="Q26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U26" s="10" t="n">
-        <v>36</v>
+      <c r="Q26" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="R26" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="S26" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="T26" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="U26" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="V26" s="10" t="n">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="W26" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="X26" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="X26" s="10" t="n">
+      <c r="Y26" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z26" s="10" t="n">
         <v>5</v>
-      </c>
-      <c r="Y26" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="Z26" s="10" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
@@ -2805,27 +2683,27 @@
         </is>
       </c>
       <c r="I27" s="14" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="J27" s="14" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="K27" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L27" s="14" t="n">
-        <v>6</v>
+        <v>3</v>
+      </c>
+      <c r="L27" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="M27" s="14" t="n">
         <v>3</v>
       </c>
       <c r="N27" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="O27" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="O27" s="14" t="n">
+        <v>43</v>
       </c>
       <c r="P27" s="14" t="n">
         <v>19</v>
@@ -2842,31 +2720,23 @@
       <c r="T27" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="U27" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U27" s="14" t="n">
+        <v>26</v>
       </c>
       <c r="V27" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="W27" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X27" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y27" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>17</v>
+      </c>
+      <c r="W27" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="X27" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Y27" s="14" t="n">
+        <v>3</v>
       </c>
       <c r="Z27" s="14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
@@ -2907,22 +2777,22 @@
         </is>
       </c>
       <c r="I28" s="10" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="J28" s="10" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="K28" s="10" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M28" s="10" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N28" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="O28" s="15" t="inlineStr">
         <is>
@@ -2935,22 +2805,22 @@
       <c r="S28" s="16" t="n"/>
       <c r="T28" s="16" t="n"/>
       <c r="U28" s="10" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="V28" s="10" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="W28" s="10" t="n">
         <v>0</v>
       </c>
       <c r="X28" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Z28" s="10" t="n">
         <v>4</v>
-      </c>
-      <c r="Y28" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="Z28" s="10" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="29" ht="28" customHeight="1">
@@ -2990,35 +2860,25 @@
           <t>ヒューストン大出身、シックスマンの3&amp;Dガード</t>
         </is>
       </c>
-      <c r="I29" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J29" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K29" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I29" s="14" t="n">
+        <v>22</v>
+      </c>
+      <c r="J29" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="K29" s="14" t="n">
+        <v>2</v>
       </c>
       <c r="L29" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M29" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N29" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M29" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="N29" s="14" t="n">
+        <v>2</v>
       </c>
       <c r="O29" s="14" t="n">
         <v>24</v>
@@ -3038,25 +2898,33 @@
       <c r="T29" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="U29" s="14" t="n">
-        <v>22</v>
+      <c r="U29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="V29" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="W29" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="W29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="X29" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y29" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z29" s="14" t="n">
-        <v>2</v>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Y29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Z29" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
     </row>
     <row r="30" ht="28" customHeight="1">
@@ -3096,34 +2964,28 @@
           <t>コネチカット大出身、ベテラン控えC、リバウンド職人</t>
         </is>
       </c>
-      <c r="I30" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I30" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="J30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K30" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L30" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="M30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O30" s="10" t="n">
@@ -3140,18 +3002,20 @@
       </c>
       <c r="S30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="T30" s="10" t="n">
         <v>8</v>
       </c>
-      <c r="U30" s="10" t="n">
-        <v>15</v>
+      <c r="U30" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="V30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="W30" s="10" t="n">
@@ -3162,12 +3026,12 @@
       </c>
       <c r="Y30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Z30" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3208,88 +3072,50 @@
           <t>ケンタッキー大出身、2年目のフォワードでローテ要員</t>
         </is>
       </c>
-      <c r="I31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O31" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="P31" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="J31" s="18" t="n"/>
+      <c r="K31" s="18" t="n"/>
+      <c r="L31" s="18" t="n"/>
+      <c r="M31" s="18" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="17" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="P31" s="18" t="n"/>
+      <c r="Q31" s="18" t="n"/>
+      <c r="R31" s="18" t="n"/>
+      <c r="S31" s="18" t="n"/>
+      <c r="T31" s="18" t="n"/>
       <c r="U31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V31" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="W31" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="W31" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="X31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Y31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Z31" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3331,11 +3157,11 @@
         </is>
       </c>
       <c r="I32" s="10" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="K32" s="10" t="n">
@@ -3346,12 +3172,12 @@
       </c>
       <c r="M32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="O32" s="10" t="n">
@@ -3372,32 +3198,24 @@
       <c r="T32" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="U32" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="U32" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="V32" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="W32" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X32" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y32" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="W32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="10" t="n">
+        <v>0</v>
       </c>
       <c r="Z32" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3438,72 +3256,82 @@
           <t>今季ツーウェイから本契約昇格、ハッスル系フォワード</t>
         </is>
       </c>
-      <c r="I33" s="17" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="J33" s="18" t="n"/>
-      <c r="K33" s="18" t="n"/>
-      <c r="L33" s="18" t="n"/>
-      <c r="M33" s="18" t="n"/>
-      <c r="N33" s="18" t="n"/>
-      <c r="O33" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P33" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q33" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R33" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="I33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N33" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O33" s="14" t="n">
+        <v>16</v>
+      </c>
+      <c r="P33" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q33" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="S33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T33" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="T33" s="14" t="n">
+        <v>2</v>
       </c>
       <c r="U33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V33" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="X33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Y33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Z33" s="14" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3544,49 +3372,65 @@
           <t>LSU出身、夏に加入のスケールあるベンチPF</t>
         </is>
       </c>
-      <c r="I34" s="15" t="inlineStr">
-        <is>
-          <t>DNP</t>
-        </is>
-      </c>
-      <c r="J34" s="16" t="n"/>
-      <c r="K34" s="16" t="n"/>
-      <c r="L34" s="16" t="n"/>
-      <c r="M34" s="16" t="n"/>
-      <c r="N34" s="16" t="n"/>
+      <c r="I34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N34" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="O34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P34" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P34" s="10" t="n">
+        <v>1</v>
       </c>
       <c r="Q34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="R34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="S34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="T34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="U34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="V34" s="10" t="n">
@@ -3594,130 +3438,112 @@
       </c>
       <c r="W34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="X34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Y34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
       <c r="Z34" s="10" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="11" t="n">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>キャメロン・ペイン</t>
+          <t>デイレン・テリー</t>
         </is>
       </c>
       <c r="C35" s="11" t="inlineStr">
         <is>
-          <t>PG</t>
+          <t>SG</t>
         </is>
       </c>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>188cm</t>
+          <t>198cm</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>84kg</t>
+          <t>88kg</t>
         </is>
       </c>
       <c r="F35" s="11" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
-          <t>11年目</t>
+          <t>4年目</t>
         </is>
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
-          <t>マレーシア州立大出身、ベテランPG、シーズン途中復帰</t>
-        </is>
-      </c>
-      <c r="I35" s="17" t="inlineStr">
+          <t>アリゾナ大出身。4月にPaynは契約解除→本契約に昇格</t>
+        </is>
+      </c>
+      <c r="I35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="N35" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O35" s="17" t="inlineStr">
         <is>
           <t>DNP</t>
         </is>
       </c>
-      <c r="J35" s="18" t="n"/>
-      <c r="K35" s="18" t="n"/>
-      <c r="L35" s="18" t="n"/>
-      <c r="M35" s="18" t="n"/>
-      <c r="N35" s="18" t="n"/>
-      <c r="O35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V35" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="W35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z35" s="14" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="P35" s="18" t="n"/>
+      <c r="Q35" s="18" t="n"/>
+      <c r="R35" s="18" t="n"/>
+      <c r="S35" s="18" t="n"/>
+      <c r="T35" s="18" t="n"/>
+      <c r="U35" s="17" t="inlineStr">
+        <is>
+          <t>DNP</t>
+        </is>
+      </c>
+      <c r="V35" s="18" t="n"/>
+      <c r="W35" s="18" t="n"/>
+      <c r="X35" s="18" t="n"/>
+      <c r="Y35" s="18" t="n"/>
+      <c r="Z35" s="18" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="7" t="n">
@@ -3753,7 +3579,7 @@
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>オーバーン大出身、2巡指名ルーキー、メニスカス手術明け</t>
+          <t>オーバーン大出身、2巡指名ルーキー、半月板手術明け</t>
         </is>
       </c>
       <c r="I36" s="15" t="inlineStr">
@@ -3788,38 +3614,36 @@
       <c r="Z36" s="16" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="U16:Z16"/>
+  <mergeCells count="30">
+    <mergeCell ref="I7:N7"/>
     <mergeCell ref="I22:N22"/>
+    <mergeCell ref="O35:T35"/>
     <mergeCell ref="I18:N18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="I3:N3"/>
     <mergeCell ref="O22:T22"/>
-    <mergeCell ref="U7:Z7"/>
+    <mergeCell ref="O31:T31"/>
     <mergeCell ref="U3:Z3"/>
     <mergeCell ref="O16:T16"/>
-    <mergeCell ref="I33:N33"/>
     <mergeCell ref="A1:Z1"/>
-    <mergeCell ref="U18:Z18"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="I17:N17"/>
     <mergeCell ref="O17:T17"/>
-    <mergeCell ref="I35:N35"/>
     <mergeCell ref="I19:N19"/>
     <mergeCell ref="U19:Z19"/>
     <mergeCell ref="A21:Z21"/>
+    <mergeCell ref="I31:N31"/>
+    <mergeCell ref="U35:Z35"/>
     <mergeCell ref="A2:Z2"/>
-    <mergeCell ref="I34:N34"/>
     <mergeCell ref="O3:T3"/>
     <mergeCell ref="U22:Z22"/>
-    <mergeCell ref="O19:T19"/>
+    <mergeCell ref="I15:N15"/>
     <mergeCell ref="O10:T10"/>
     <mergeCell ref="O28:T28"/>
     <mergeCell ref="O18:T18"/>
     <mergeCell ref="I36:N36"/>
     <mergeCell ref="O36:T36"/>
     <mergeCell ref="U36:Z36"/>
-    <mergeCell ref="U17:Z17"/>
     <mergeCell ref="I16:N16"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>

</xml_diff>